<commit_message>
NPB自動更新(2軍): 2026-10-03 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/2軍/公式戦/raw/2026-10-03/highlights_20261003.xlsx
+++ b/data/プロ野球/2026年/2軍/公式戦/raw/2026-10-03/highlights_20261003.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>8回裏に勝ち越しのタイムリースリーベースを放ち、チームを勝利に導いた。</t>
+          <t>8回裏、二死二塁から勝ち越しのタイムリースリーベースを放ち、チームを勝利に導いた。</t>
         </is>
       </c>
     </row>
@@ -504,17 +504,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>三方 陽登</t>
+          <t>下川 隼佑</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>オリックス</t>
+          <t>ヤクルト</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>6回裏に逆転タイムリーヒットを放ち、試合の流れを大きく変えた。</t>
+          <t>先発として6回を投げ、わずか1失点に抑える好投で試合を作り、勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -529,17 +529,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>下川 隼佑</t>
+          <t>三方 陽登</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ヤクルト</t>
+          <t>オリックス</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>先発として6回を投げ1失点と好投し、チームの勝利に貢献した。</t>
+          <t>6回裏、二死二三塁のチャンスでライトへ逆転タイムリーを放ち、試合の流れを変えた。</t>
         </is>
       </c>
     </row>
@@ -554,17 +554,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>澤井 廉</t>
+          <t>植田 将太</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ヤクルト</t>
+          <t>ロッテ</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>5打数3安打の猛打賞を記録し、打線の中核として活躍を見せた。</t>
+          <t>2回表にランナー二塁からレフトへ逆転タイムリーツーベースを放ち、チームを勢いづけた。</t>
         </is>
       </c>
     </row>
@@ -579,17 +579,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>漆原 幻汰</t>
+          <t>横田 蒼和</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>オイシックス</t>
+          <t>西武</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5打数3安打の猛打賞で、チームの攻撃を牽引する活躍だった。</t>
+          <t>4回表、二死三塁からレフトへ先制タイムリーヒットを放ち、チームに貴重な1点をもたらした。</t>
         </is>
       </c>
     </row>

</xml_diff>